<commit_message>
excelsheet contain 2 sheet,fetching data from second for 2 website.
</commit_message>
<xml_diff>
--- a/src/test/java/ExcelDataForMultiple/Rediff Data.xlsx
+++ b/src/test/java/ExcelDataForMultiple/Rediff Data.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0368638-9739-432F-BF95-CFFB37D90B3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCD48B3F-FB93-4EEA-B43D-95DF2BE2E93A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
+    <sheet name="SauceLoginusernames" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="19">
   <si>
     <t>testUser1</t>
   </si>
@@ -58,6 +59,30 @@
   </si>
   <si>
     <t>password</t>
+  </si>
+  <si>
+    <t>usernames</t>
+  </si>
+  <si>
+    <t>standard_user</t>
+  </si>
+  <si>
+    <t>secret_sauce</t>
+  </si>
+  <si>
+    <t>locked_out_user</t>
+  </si>
+  <si>
+    <t>problem_user</t>
+  </si>
+  <si>
+    <t>performance_glitch_user</t>
+  </si>
+  <si>
+    <t>error_user</t>
+  </si>
+  <si>
+    <t>visual_user</t>
   </si>
 </sst>
 </file>
@@ -440,4 +465,74 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0560C776-E1BB-47B2-A512-546CCC068052}">
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="21.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.54296875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>